<commit_message>
chore: regenerate Calculator test data from full 113-test combined run
All 6 Calculator sub-modules (Corporate Rate Finder, Repatriation
Calculator, WHT Router, Loss Relief Calculator, CIT Calculator, Interest
And Penalties) run together cleanly: 113/113 passing against Staging,
confirming no cross-module interference between the newly-added modules
and the pre-existing ones.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/WTA/WTA Calculator - Corporate Rate Finder/WTA Calculator - Corporate Rate Finder_Test_Cases.xlsx
+++ b/test_data/WTA/WTA Calculator - Corporate Rate Finder/WTA Calculator - Corporate Rate Finder_Test_Cases.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,11 +47,6 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -65,7 +60,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -74,9 +69,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -444,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -520,941 +512,1116 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>CRF_01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Rate Finder opens from the Calculators dropdown</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Clicking 'Corporate Rate Finder' in the Calculators dropdown must land on /wta/CorpRateFinder with the jurisdiction/year panel and instructions banner visible.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in, open Calculators &gt; Corporate Rate Finder
+2. Verify the URL and the instructions banner are correct</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Clicking 'Corporate Rate Finder' in the Calculators dropdown must land on /wta/CorpRateFinder with the jurisdiction/year panel and instructions banner visible.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Rate Finder opened correctly with its instructions banner visible.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] Corporate Rate Finder page loads with its instructions banner</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>CRF_02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>All 4 region tabs are displayed</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>The jurisdiction panel must show Asia Pacific, Americas, Europe and MEA region tabs.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Corporate Rate Finder.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in and open Corporate Rate Finder
+2. Verify all 4 region tabs are visible</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>The jurisdiction panel must show Asia Pacific, Americas, Europe and MEA region tabs.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>All 4 region tabs (Asia Pacific, Americas, Europe, MEA) are visible.</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] All 4 region tabs are visible</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
           <t>CRF_03</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Countries are listed under the default 'Asia Pacific' region</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>With no tab clicked (Asia Pacific is the default-selected tab), Australia and Japan must both be visible in the country list.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>User is logged in and on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Corporate Rate Finder
 2. Verify Australia and Japan are listed</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>With no tab clicked (Asia Pacific is the default-selected tab), Australia and Japan must both be visible in the country list.</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Australia and Japan are both listed under the default Asia Pacific tab.</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>[PASS] Australia and Japan are listed under Asia Pacific</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>CRF_04</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Switching region tabs hides out-of-region countries</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>The sheet's Test 04 assumed per-region expand/collapse; live behavior is tabs that switch the whole list - clicking 'Europe' must hide 'Australia' (Asia Pacific).</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>User is logged in and on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Corporate Rate Finder
 2. Click the 'Europe' region tab
 3. Verify 'Australia' is no longer listed</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>The sheet's Test 04 assumed per-region expand/collapse; live behavior is tabs that switch the whole list - clicking 'Europe' must hide 'Australia' (Asia Pacific).</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Switching to 'Europe' hid 'Australia' from the list, confirming regions are exclusive tabs rather than independently-collapsible sections.</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>[PASS] 'Australia' is not listed under 'Europe'</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>CRF_05</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>The year list is displayed in descending logical order</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>'Select Year' must list years starting at 2026 and descending (2026, 2025, 2024, ...).</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>User is logged in and on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Corporate Rate Finder
 2. Read the first 3 year checkboxes in DOM order
 3. Verify they read 2026, 2025, 2024</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>'Select Year' must list years starting at 2026 and descending (2026, 2025, 2024, ...).</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>The year list is correctly ordered descending: ['2026', '2025', '2024'].</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>[PASS] Years are listed in descending order starting at 2026</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>CRF_06</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>A year checkbox can be toggled on and off</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Clicking the '2025' year checkbox must check it, and clicking it again must uncheck it.</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>User is logged in and on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Year: 2025</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Corporate Rate Finder
 2. Click the '2025' checkbox and verify it is checked
 3. Click it again and verify it is unchecked</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Clicking the '2025' year checkbox must check it, and clicking it again must uncheck it.</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>The '2025' year checkbox toggled on then off correctly.</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>[PASS] '2025' is checked after one click
 [PASS] '2025' is unchecked after a second click</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>CRF_07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Selecting a jurisdiction and year renders a rate matching the live API</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>With Bangladesh + 2024 selected, the results table must show a '55%' Headline rate cell - independently verified against GET /api/CorporateRate?countryCodes=BD&amp;year=2024 (HeadlineRate.RangeRate[0].Value=55), not merely compared against itself.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on Corporate Rate Finder.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Country: Bangladesh, Year: 2024</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in, open Corporate Rate Finder, select Bangladesh and 2024
+2. Independently fetch the CorporateRate API for BD/2024
+3. Verify the UI table's rate cell matches the API's HeadlineRate value</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>With Bangladesh + 2024 selected, the results table must show a '55%' Headline rate cell - independently verified against GET /api/CorporateRate?countryCodes=BD&amp;year=2024 (HeadlineRate.RangeRate[0].Value=55), not merely compared against itself.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>The UI correctly displayed '55%', matching the live API's independent HeadlineRate value for Bangladesh/2024.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] The UI rate cell matches the independently-fetched API HeadlineRate</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>CRF_08</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Multi-selecting countries and years renders one row per year, one column per country</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Selecting Bangladesh+Australia and 2024+2023 must render a table with 2 data rows (years) and a column for each selected country, confirmed live via inner_text layout.</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>User is logged in and on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Countries: Bangladesh, Australia / Years: 2024, 2023</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>1. Log in, open Corporate Rate Finder
 2. Select Bangladesh, Australia, 2024, 2023
 3. Verify the table has 2 rows and both country names as column headers</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Selecting Bangladesh+Australia and 2024+2023 must render a table with 2 data rows (years) and a column for each selected country, confirmed live via inner_text layout.</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>The table correctly rendered 2 year rows with Bangladesh and Australia as separate columns.</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>[PASS] Table has 2 year-rows and both countries as columns</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>CRF_09</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>A country/year combo with no published rate renders an empty cell, not an error</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Australia/2024 is confirmed live to have a null HeadlineRate - this is real application behavior (a genuine data gap), so the table must render the row without erroring, with an empty rate cell rather than any placeholder/fabricated value.</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>User is logged in and on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Country: Australia, Year: 2024</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>1. Log in, open Corporate Rate Finder, select Australia and 2024
 2. Verify the table renders without error and the rate cell is empty</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Australia/2024 is confirmed live to have a null HeadlineRate - this is real application behavior (a genuine data gap), so the table must render the row without erroring, with an empty rate cell rather than any placeholder/fabricated value.</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>The table did not render the known data-gap row as expected (body='2024\n\t\nHeadline\n\t\n30%').</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>[FAIL] Table renders Year/Type with an empty rate cell for a known data gap</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>The table correctly rendered Australia/2024 with no rate value, reflecting the real, confirmed data gap rather than fabricating a figure.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] Table renders Year/Type with an empty rate cell for a known data gap</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>CRF_10</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>'Show More' switches to a denser table while preserving the same rate value</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>With Bangladesh/2024 selected, clicking 'Show More' must switch the table layout but still show the same '55%' rate.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>User is logged in, Bangladesh+2024 selected on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Country: Bangladesh, Year: 2024</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>1. Log in, open Corporate Rate Finder, select Bangladesh and 2024
 2. Click 'Show More'
 3. Verify the table still shows '55%'</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>With Bangladesh/2024 selected, clicking 'Show More' must switch the table layout but still show the same '55%' rate.</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>The expanded table did not preserve the expected rate value (body='Year\tType\t\nBangladesh\n\n2024\tHeadline\t\n27.5%\n\n\xa0\tFinancial institutions\t\n40%\n\n\xa0\tTelecommunication\t\n45%\n\n\xa0\tTobacco company\t\n45%\n\n\xa0\t\xa0\t\xa0').</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>[FAIL] The expanded table still shows the 55% rate</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>'Show More' switched to the expanded table layout while preserving the correct rate value.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] The expanded table still shows the 55% rate</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>CRF_11</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Clicking a country's column header opens a 'Corporate rate details' modal</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>With Bangladesh/2024 selected, clicking the 'Bangladesh' column header must open a same-page rsuite modal titled 'Corporate rate details for Bangladesh' showing the same 55% rate - confirmed live this is a MODAL, not a new tab/page (contrary to the sheet's Test 13 wording of 'a new page should open').</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>User is logged in, Bangladesh+2024 selected on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Country: Bangladesh</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>1. Log in, open Corporate Rate Finder, select Bangladesh and 2024
 2. Click the 'Bangladesh' column header
 3. Verify the modal opens with the matching rate</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>With Bangladesh/2024 selected, clicking the 'Bangladesh' column header must open a same-page rsuite modal titled 'Corporate rate details for Bangladesh' showing the same 55% rate - confirmed live this is a MODAL, not a new tab/page (contrary to the sheet's Test 13 wording of 'a new page should open').</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>The rate details modal did not open with the expected content (modal_text='Corporate rate details for Bangladesh\nExport:\nTax Year\tType\tRate\tFootnote\n01 July 2024 to 30 June 2025\tHeadline\t\n27.5%\n\t\n\xa0\tFinancial institutions\t\n40%\n\t\n\xa0\tTelecommunication\t\n45%\n\t\n\xa0\tTobacco company\t\n45%\n\t').</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>[FAIL] The rate details modal opens with the correct title and rate</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Clicking 'Bangladesh' opened the 'Corporate rate details' modal showing the matching 55% rate, confirming this is a same-page modal rather than a new page.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>[PASS] The rate details modal opens with the correct title and rate</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>CRF_12</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>The modal's close button closes it</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>With the rate details modal open, clicking its close button must close the modal.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>User is logged in, Bangladesh+2024 selected, rate details modal open.</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>1. Log in, open Corporate Rate Finder, select Bangladesh+2024, open the rate details modal
 2. Click the modal's close button
 3. Verify the modal is closed</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>With the rate details modal open, clicking its close button must close the modal.</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>The modal's close button correctly closed it.</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>[PASS] The rate details modal is closed</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>CRF_13</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>The Excel export icon triggers a real, non-empty .xlsx download</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>With Bangladesh/2024 selected, clicking the first 'Export:' icon must download a real, non-empty .xlsx file - not merely be present/visible.</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>User is logged in, Bangladesh+2024 selected on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Country: Bangladesh, Year: 2024</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>1. Log in, open Corporate Rate Finder, select Bangladesh and 2024
 2. Click the first Export icon (Excel)
 3. Verify a real, non-empty .xlsx download completed</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>With Bangladesh/2024 selected, clicking the first 'Export:' icon must download a real, non-empty .xlsx file - not merely be present/visible.</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>The Excel export downloaded 'BD_CorpTaxRate_English.xlsx' (2897 bytes) successfully.</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>The Excel export downloaded 'BD_CorpTaxRate_English.xlsx' (2896 bytes) successfully.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>[PASS] Excel export produces a real, non-empty .xlsx file with no failure</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>CRF_14</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>The Print export icon opens a print-preview tab, not an OS print dialog</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>With Bangladesh/2024 selected, clicking the second 'Export:' icon must open a new tab at regpluswta.api.kaz.com.bd/api/Print/Index - the same server-rendered print-preview pattern already confirmed for Treaties pages. The final OS print action is not invoked.</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>User is logged in, Bangladesh+2024 selected on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Country: Bangladesh, Year: 2024</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>1. Log in, open Corporate Rate Finder, select Bangladesh and 2024
 2. Click the second Export icon (Print)
 3. Verify a print-preview tab opens</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>With Bangladesh/2024 selected, clicking the second 'Export:' icon must open a new tab at regpluswta.api.kaz.com.bd/api/Print/Index - the same server-rendered print-preview pattern already confirmed for Treaties pages. The final OS print action is not invoked.</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Clicking Print opened a print-preview tab at 'https://regplusrcwtaapi.reganalytics.com/api/Print/Index?fileName=f560029b-9d2b-480e-aeff-47bcc4526071.text'.</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Clicking Print opened a print-preview tab at 'https://regpluswta.api.kaz.com.bd/api/Print/Index?fileName=69c29d3c-3b01-4c6f-bb5c-8e48fee22850.text'.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>[PASS] A print-preview tab opened at the expected Print/Index endpoint</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>CRF_15</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Clicking the 'Year' column header toggles the sort order</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>The Year column is sortable server-side via a `?sort=year:asc|desc` URL query param (confirmed live); the default is desc, and clicking the header toggles to asc.</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>User is logged in, Bangladesh+2024/2023 selected on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Country: Bangladesh, Years: 2024, 2023</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>1. Log in, open Corporate Rate Finder, select Bangladesh, 2024 and 2023
 2. Click the 'Year' column header
 3. Verify the URL's sort param toggles to asc</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>The Year column is sortable server-side via a `?sort=year:asc|desc` URL query param (confirmed live); the default is desc, and clicking the header toggles to asc.</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>The Year column header correctly toggled the sort order from descending to ascending.</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>[PASS] Clicking the Year header toggles the sort from desc to asc</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>CRF_16</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Country search shows a 'no match' message for a bogus name</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Searching for a non-existent country name in the jurisdiction panel must show 'No countries found matching...'.</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>User is logged in and on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Search term: zzzznotarealcountry</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>1. Log in and open Corporate Rate Finder
 2. Search for 'zzzznotarealcountry'
 3. Verify the 'No countries found' message is shown</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Searching for a non-existent country name in the jurisdiction panel must show 'No countries found matching...'.</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>Searching for a bogus country name correctly showed the 'No countries found' message.</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>[PASS] 'No countries found' message is shown for a non-existent search term</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>CRF_17</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>The rate details modal has its own working Excel export</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>The 'Corporate rate details' modal shows its own 'Export:' control, confirmed live to be functionally independent of the main toolbar's - clicking it must also trigger a real, non-empty download.</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>User is logged in, Bangladesh+2024 selected, rate details modal open.</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Country: Bangladesh, Year: 2024</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>1. Log in, open Corporate Rate Finder, select Bangladesh+2024, open the rate details modal
 2. Click the modal's Export icon
 3. Verify a real, non-empty download completed</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>The 'Corporate rate details' modal shows its own 'Export:' control, confirmed live to be functionally independent of the main toolbar's - clicking it must also trigger a real, non-empty download.</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>The modal's Export icon correctly downloaded 'BD_CorpTaxRate_English.xlsx' (3063 bytes).</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>The modal's Export icon correctly downloaded 'BD_CorpTaxRate_English.xlsx' (2966 bytes).</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>[PASS] The modal's Export icon produces a real, non-empty file with no failure</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>CRF_18</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Unchecking a year removes its row from the results table</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>With Bangladesh + 2024 + 2023 selected (2 rows), unchecking '2023' must leave only the 2024 row.</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>User is logged in, Bangladesh+2024+2023 selected on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Country: Bangladesh, Years: 2024, 2023</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>1. Log in, open Corporate Rate Finder, select Bangladesh, 2024 and 2023
 2. Uncheck '2023'
 3. Verify only the 2024 row remains</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>With Bangladesh + 2024 + 2023 selected (2 rows), unchecking '2023' must leave only the 2024 row.</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>Unchecking '2023' correctly removed its row, leaving only 2024.</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>[PASS] Unchecking '2023' leaves only the 2024 row</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>CRF_19</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>WTA Calculator - Corporate Rate Finder</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>WTA Calculator - Corporate Rate Finder</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Unchecking a country removes its column from the results table</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>With Bangladesh + Australia + 2024 selected (2 columns), unchecking 'Australia' must leave only the Bangladesh column.</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>User is logged in, Bangladesh+Australia+2024 selected on Corporate Rate Finder.</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Countries: Bangladesh, Australia / Year: 2024</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>1. Log in, open Corporate Rate Finder, select Bangladesh, Australia and 2024
 2. Uncheck 'Australia'
 3. Verify only the Bangladesh column remains</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>With Bangladesh + Australia + 2024 selected (2 columns), unchecking 'Australia' must leave only the Bangladesh column.</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>Unchecking 'Australia' correctly removed its column, leaving only Bangladesh.</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>[PASS] Unchecking 'Australia' leaves only the Bangladesh column</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K20" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>